<commit_message>
Update concept and Gantt
</commit_message>
<xml_diff>
--- a/Theory/Gantt_Franzelin.xlsx
+++ b/Theory/Gantt_Franzelin.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\Master-Thesis-GEOAI\Theory\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0420FB90-46EA-464D-9574-72F25591B919}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C70A86B-B36C-4826-853E-E9B63CAD5067}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -188,9 +188,6 @@
     <t>Evaluation &amp; Application Case</t>
   </si>
   <si>
-    <t>Writing (Results, Discussion, Conclusion)</t>
-  </si>
-  <si>
     <t>Finalization</t>
   </si>
   <si>
@@ -254,14 +251,17 @@
     <t>M7</t>
   </si>
   <si>
-    <t>M9</t>
+    <t>M8</t>
+  </si>
+  <si>
+    <t>Writing</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -377,6 +377,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="12">
     <fill>
@@ -949,7 +955,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1181,6 +1187,9 @@
     </xf>
     <xf numFmtId="14" fontId="14" fillId="2" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1508,7 +1517,7 @@
   <sheetData>
     <row r="1" spans="2:51" s="9" customFormat="1" ht="36.75" thickBot="1" x14ac:dyDescent="0.6">
       <c r="B1" s="77" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" spans="2:51" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1882,7 +1891,7 @@
       <c r="H5" s="40"/>
       <c r="I5" s="36"/>
       <c r="J5" s="68" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="K5" s="50"/>
       <c r="L5" s="50"/>
@@ -1891,12 +1900,12 @@
       <c r="O5" s="27"/>
       <c r="P5" s="27"/>
       <c r="Q5" s="68" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="R5" s="27"/>
       <c r="S5" s="28"/>
       <c r="T5" s="68" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="U5" s="28"/>
       <c r="V5" s="59"/>
@@ -1906,7 +1915,7 @@
       <c r="Z5" s="27"/>
       <c r="AA5" s="27"/>
       <c r="AB5" s="68" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="AC5" s="28"/>
       <c r="AD5" s="28"/>
@@ -1914,25 +1923,25 @@
       <c r="AF5" s="27"/>
       <c r="AG5" s="28"/>
       <c r="AH5" s="68" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="AI5" s="27"/>
       <c r="AJ5" s="27"/>
       <c r="AK5" s="59"/>
       <c r="AL5" s="28"/>
       <c r="AM5" s="68" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="AN5" s="28"/>
       <c r="AO5" s="27"/>
       <c r="AP5" s="68" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="AQ5" s="28"/>
       <c r="AR5" s="28"/>
       <c r="AS5" s="28"/>
       <c r="AT5" s="68" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AU5"/>
       <c r="AV5"/>
@@ -2052,11 +2061,11 @@
       <c r="B8" s="24"/>
       <c r="C8" s="25"/>
       <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
+      <c r="E8" s="80"/>
       <c r="F8" s="5"/>
       <c r="G8" s="5"/>
-      <c r="H8" s="41"/>
-      <c r="I8" s="37"/>
+      <c r="H8" s="5"/>
+      <c r="I8" s="5"/>
       <c r="J8" s="48"/>
       <c r="K8" s="44"/>
       <c r="L8" s="44"/>
@@ -2269,7 +2278,7 @@
       <c r="G12" s="71"/>
       <c r="H12" s="72"/>
       <c r="I12" s="72"/>
-      <c r="J12" s="55"/>
+      <c r="J12" s="72"/>
       <c r="K12" s="73"/>
       <c r="L12" s="73"/>
       <c r="M12" s="55"/>
@@ -2280,14 +2289,14 @@
       <c r="R12" s="69"/>
       <c r="S12" s="75"/>
       <c r="T12" s="75"/>
-      <c r="U12" s="75"/>
+      <c r="U12" s="55"/>
       <c r="V12" s="76"/>
       <c r="W12" s="75"/>
       <c r="X12" s="75"/>
       <c r="Y12" s="73"/>
       <c r="Z12" s="69"/>
       <c r="AA12" s="69"/>
-      <c r="AB12" s="75"/>
+      <c r="AB12" s="55"/>
       <c r="AC12" s="75"/>
       <c r="AD12" s="75"/>
       <c r="AE12" s="75"/>
@@ -2472,7 +2481,7 @@
     </row>
     <row r="16" spans="2:51" s="13" customFormat="1" ht="45.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="66" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C16" s="18"/>
       <c r="D16" s="19"/>
@@ -2527,8 +2536,8 @@
     <row r="17" spans="2:51" s="13" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="24"/>
       <c r="C17" s="25"/>
-      <c r="D17" s="21"/>
-      <c r="E17" s="21"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
       <c r="F17" s="21"/>
       <c r="G17" s="21"/>
       <c r="H17" s="41"/>
@@ -2684,7 +2693,7 @@
     </row>
     <row r="20" spans="2:51" s="13" customFormat="1" ht="40.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B20" s="66" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C20" s="18"/>
       <c r="D20" s="19"/>
@@ -2896,7 +2905,7 @@
     </row>
     <row r="24" spans="2:51" s="13" customFormat="1" ht="53.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B24" s="66" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C24" s="18"/>
       <c r="D24" s="19"/>
@@ -3108,7 +3117,7 @@
     </row>
     <row r="28" spans="2:51" s="13" customFormat="1" ht="53.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B28" s="66" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C28" s="18"/>
       <c r="D28" s="19"/>
@@ -3141,10 +3150,10 @@
       <c r="AE28" s="19"/>
       <c r="AF28" s="20"/>
       <c r="AG28" s="20"/>
-      <c r="AH28" s="20"/>
-      <c r="AI28" s="61"/>
-      <c r="AJ28" s="20"/>
-      <c r="AK28" s="20"/>
+      <c r="AH28" s="55"/>
+      <c r="AI28" s="55"/>
+      <c r="AJ28" s="55"/>
+      <c r="AK28" s="55"/>
       <c r="AL28" s="19"/>
       <c r="AM28" s="19"/>
       <c r="AN28" s="19"/>
@@ -3534,9 +3543,9 @@
       <c r="AX35"/>
       <c r="AY35"/>
     </row>
-    <row r="36" spans="2:51" s="13" customFormat="1" ht="53.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:51" s="13" customFormat="1" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B36" s="66" t="s">
-        <v>50</v>
+        <v>72</v>
       </c>
       <c r="C36" s="18"/>
       <c r="D36" s="19"/>
@@ -3748,7 +3757,7 @@
     </row>
     <row r="40" spans="2:51" s="13" customFormat="1" ht="45.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B40" s="66" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C40" s="18"/>
       <c r="D40" s="19"/>
@@ -4122,7 +4131,7 @@
     </row>
     <row r="47" spans="2:51" s="13" customFormat="1" ht="53.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B47" s="66" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C47"/>
       <c r="D47"/>
@@ -4191,63 +4200,63 @@
     </row>
     <row r="56" spans="4:32" ht="30" x14ac:dyDescent="0.25">
       <c r="D56" s="67" t="s">
+        <v>53</v>
+      </c>
+      <c r="E56" s="67" t="s">
         <v>54</v>
-      </c>
-      <c r="E56" s="67" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="57" spans="4:32" ht="75" x14ac:dyDescent="0.25">
       <c r="D57" s="65" t="s">
+        <v>51</v>
+      </c>
+      <c r="E57" s="64" t="s">
         <v>52</v>
-      </c>
-      <c r="E57" s="64" t="s">
-        <v>53</v>
       </c>
       <c r="AF57"/>
     </row>
     <row r="58" spans="4:32" ht="60" x14ac:dyDescent="0.25">
       <c r="D58" s="65" t="s">
+        <v>55</v>
+      </c>
+      <c r="E58" s="64" t="s">
         <v>56</v>
-      </c>
-      <c r="E58" s="64" t="s">
-        <v>57</v>
       </c>
       <c r="AF58"/>
     </row>
     <row r="59" spans="4:32" ht="45" x14ac:dyDescent="0.25">
       <c r="D59" s="65" t="s">
+        <v>57</v>
+      </c>
+      <c r="E59" s="64" t="s">
         <v>58</v>
-      </c>
-      <c r="E59" s="64" t="s">
-        <v>59</v>
       </c>
       <c r="AF59"/>
     </row>
     <row r="60" spans="4:32" ht="60" x14ac:dyDescent="0.25">
       <c r="D60" s="65" t="s">
+        <v>59</v>
+      </c>
+      <c r="E60" s="64" t="s">
         <v>60</v>
-      </c>
-      <c r="E60" s="64" t="s">
-        <v>61</v>
       </c>
       <c r="AF60"/>
     </row>
     <row r="61" spans="4:32" ht="60" x14ac:dyDescent="0.25">
       <c r="D61" s="65" t="s">
+        <v>61</v>
+      </c>
+      <c r="E61" s="64" t="s">
         <v>62</v>
-      </c>
-      <c r="E61" s="64" t="s">
-        <v>63</v>
       </c>
       <c r="AF61"/>
     </row>
     <row r="62" spans="4:32" ht="30" x14ac:dyDescent="0.25">
       <c r="D62" s="65" t="s">
+        <v>63</v>
+      </c>
+      <c r="E62" s="64" t="s">
         <v>64</v>
-      </c>
-      <c r="E62" s="64" t="s">
-        <v>65</v>
       </c>
       <c r="AF62"/>
     </row>

</xml_diff>